<commit_message>
read Zerodha tables starting in any column
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample-pnl.xlsx
+++ b/tests/fixtures/sample-pnl.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity P&amp;L" sheetId="1" r:id="R571b2647ed98400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account" sheetId="2" r:id="Re3e8e275959945cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equity P&amp;L" sheetId="1" r:id="Rc04fcd2e9c6a4f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account" sheetId="2" r:id="R410ae77077f4444a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -245,10 +245,10 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="str">
+      <x:c r="A1"/>
+      <x:c r="B1" t="str">
         <x:v>FAKE TEST DATA ONLY</x:v>
       </x:c>
-      <x:c r="B1"/>
       <x:c r="C1"/>
       <x:c r="D1"/>
       <x:c r="E1"/>
@@ -260,15 +260,16 @@
       <x:c r="K1"/>
       <x:c r="L1"/>
       <x:c r="M1"/>
+      <x:c r="N1"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2"/>
+      <x:c r="B2" t="str">
         <x:v>Client ID</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="C2" t="str">
         <x:v>FAKE-CLIENT-NEVER-SEND</x:v>
       </x:c>
-      <x:c r="C2"/>
       <x:c r="D2"/>
       <x:c r="E2"/>
       <x:c r="F2"/>
@@ -279,6 +280,7 @@
       <x:c r="K2"/>
       <x:c r="L2"/>
       <x:c r="M2"/>
+      <x:c r="N2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3"/>
@@ -294,15 +296,16 @@
       <x:c r="K3"/>
       <x:c r="L3"/>
       <x:c r="M3"/>
+      <x:c r="N3"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="str">
+      <x:c r="A4"/>
+      <x:c r="B4" t="str">
         <x:v>Charges</x:v>
       </x:c>
-      <x:c r="B4" t="n">
+      <x:c r="C4" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="C4"/>
       <x:c r="D4"/>
       <x:c r="E4"/>
       <x:c r="F4"/>
@@ -313,15 +316,16 @@
       <x:c r="K4"/>
       <x:c r="L4"/>
       <x:c r="M4"/>
+      <x:c r="N4"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
+      <x:c r="A5"/>
+      <x:c r="B5" t="str">
         <x:v>Other Credit &amp; Debit</x:v>
       </x:c>
-      <x:c r="B5" t="n">
+      <x:c r="C5" t="n">
         <x:v>-25</x:v>
       </x:c>
-      <x:c r="C5"/>
       <x:c r="D5"/>
       <x:c r="E5"/>
       <x:c r="F5"/>
@@ -332,15 +336,16 @@
       <x:c r="K5"/>
       <x:c r="L5"/>
       <x:c r="M5"/>
+      <x:c r="N5"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A6"/>
+      <x:c r="B6" t="str">
         <x:v>Realized P&amp;L</x:v>
       </x:c>
-      <x:c r="B6" t="n">
+      <x:c r="C6" t="n">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="C6"/>
       <x:c r="D6"/>
       <x:c r="E6"/>
       <x:c r="F6"/>
@@ -351,15 +356,16 @@
       <x:c r="K6"/>
       <x:c r="L6"/>
       <x:c r="M6"/>
+      <x:c r="N6"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="A7"/>
+      <x:c r="B7" t="str">
         <x:v>Unrealized P&amp;L</x:v>
       </x:c>
-      <x:c r="B7" t="n">
+      <x:c r="C7" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C7"/>
       <x:c r="D7"/>
       <x:c r="E7"/>
       <x:c r="F7"/>
@@ -370,6 +376,7 @@
       <x:c r="K7"/>
       <x:c r="L7"/>
       <x:c r="M7"/>
+      <x:c r="N7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8"/>
@@ -385,6 +392,7 @@
       <x:c r="K8"/>
       <x:c r="L8"/>
       <x:c r="M8"/>
+      <x:c r="N8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9"/>
@@ -400,64 +408,64 @@
       <x:c r="K9"/>
       <x:c r="L9"/>
       <x:c r="M9"/>
+      <x:c r="N9"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
+      <x:c r="A10"/>
+      <x:c r="B10" t="str">
         <x:v>Symbol</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="C10" t="str">
         <x:v>ISIN</x:v>
       </x:c>
-      <x:c r="C10" t="str">
+      <x:c r="D10" t="str">
         <x:v>Quantity</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="E10" t="str">
         <x:v>Buy Value</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="F10" t="str">
         <x:v>Sell Value</x:v>
       </x:c>
-      <x:c r="F10" t="str">
+      <x:c r="G10" t="str">
         <x:v>Realized P&amp;L</x:v>
       </x:c>
-      <x:c r="G10" t="str">
+      <x:c r="H10" t="str">
         <x:v>Realized P&amp;L Pct.</x:v>
       </x:c>
-      <x:c r="H10" t="str">
+      <x:c r="I10" t="str">
         <x:v>Previous Closing Price</x:v>
       </x:c>
-      <x:c r="I10" t="str">
+      <x:c r="J10" t="str">
         <x:v>Open Quantity</x:v>
       </x:c>
-      <x:c r="J10" t="str">
+      <x:c r="K10" t="str">
         <x:v>Open Quantity Type</x:v>
       </x:c>
-      <x:c r="K10" t="str">
+      <x:c r="L10" t="str">
         <x:v>Open Value</x:v>
       </x:c>
-      <x:c r="L10" t="str">
+      <x:c r="M10" t="str">
         <x:v>Unrealized P&amp;L</x:v>
       </x:c>
-      <x:c r="M10" t="str">
+      <x:c r="N10" t="str">
         <x:v>Unrealized P&amp;L Pct.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
+      <x:c r="A11"/>
+      <x:c r="B11" t="str">
         <x:v>FAKEALPHA</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="C11" t="str">
         <x:v>FAKEISIN0001</x:v>
       </x:c>
-      <x:c r="C11" t="n">
+      <x:c r="D11" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D11" t="n">
+      <x:c r="E11" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="E11" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="F11" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -465,40 +473,41 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" t="n">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="I11" t="n">
+      <x:c r="J11" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="J11" t="str">
+      <x:c r="K11" t="str">
         <x:v>Long</x:v>
       </x:c>
-      <x:c r="K11" t="n">
+      <x:c r="L11" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="L11" t="n">
+      <x:c r="M11" t="n">
         <x:v>5000</x:v>
       </x:c>
-      <x:c r="M11" t="n">
+      <x:c r="N11" t="n">
         <x:v>500</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="str">
+      <x:c r="A12"/>
+      <x:c r="B12" t="str">
         <x:v>FAKEBETA</x:v>
       </x:c>
-      <x:c r="B12" t="str">
+      <x:c r="C12" t="str">
         <x:v>FAKEISIN0002</x:v>
       </x:c>
-      <x:c r="C12" t="n">
+      <x:c r="D12" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="D12" t="n">
+      <x:c r="E12" t="n">
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="E12" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="F12" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -506,40 +515,41 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="I12" t="n">
+      <x:c r="J12" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="J12" t="str">
+      <x:c r="K12" t="str">
         <x:v>Long</x:v>
       </x:c>
-      <x:c r="K12" t="n">
+      <x:c r="L12" t="n">
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="L12" t="n">
+      <x:c r="M12" t="n">
         <x:v>-5000</x:v>
       </x:c>
-      <x:c r="M12" t="n">
+      <x:c r="N12" t="n">
         <x:v>-50</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
+      <x:c r="A13"/>
+      <x:c r="B13" t="str">
         <x:v>FAKEGAMMA</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="C13" t="str">
         <x:v>FAKEISIN0003</x:v>
       </x:c>
-      <x:c r="C13" t="n">
+      <x:c r="D13" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D13" t="n">
+      <x:c r="E13" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E13" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="F13" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -547,40 +557,41 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="I13" t="n">
+      <x:c r="J13" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J13" t="str">
+      <x:c r="K13" t="str">
         <x:v>Long</x:v>
       </x:c>
-      <x:c r="K13" t="n">
+      <x:c r="L13" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="L13" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="M13" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="N13" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
+      <x:c r="A14"/>
+      <x:c r="B14" t="str">
         <x:v>FAKEDELTA</x:v>
       </x:c>
-      <x:c r="B14" t="str">
+      <x:c r="C14" t="str">
         <x:v>FAKEISIN0004</x:v>
       </x:c>
-      <x:c r="C14" t="n">
+      <x:c r="D14" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D14" t="n">
+      <x:c r="E14" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="E14" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="F14" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -588,38 +599,39 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" t="n">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="I14" t="n">
+      <x:c r="J14" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J14" t="str">
+      <x:c r="K14" t="str">
         <x:v>Long</x:v>
       </x:c>
-      <x:c r="K14" t="n">
+      <x:c r="L14" t="n">
         <x:v>100</x:v>
-      </x:c>
-      <x:c r="L14" t="n">
-        <x:v>10</x:v>
       </x:c>
       <x:c r="M14" t="n">
         <x:v>10</x:v>
       </x:c>
+      <x:c r="N14" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str">
+      <x:c r="A15"/>
+      <x:c r="B15" t="str">
         <x:v>FAKEEPSILON</x:v>
       </x:c>
-      <x:c r="B15"/>
-      <x:c r="C15" t="n">
+      <x:c r="C15"/>
+      <x:c r="D15" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D15" t="n">
+      <x:c r="E15" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="E15" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="F15" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -627,37 +639,38 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="I15" t="n">
+      <x:c r="J15" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J15" t="str">
+      <x:c r="K15" t="str">
         <x:v>Long</x:v>
       </x:c>
-      <x:c r="K15" t="n">
+      <x:c r="L15" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="L15" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="M15" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="N15" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="str">
+      <x:c r="A16"/>
+      <x:c r="B16" t="str">
         <x:v>FAKEZETA</x:v>
       </x:c>
-      <x:c r="B16" t="str">
+      <x:c r="C16" t="str">
         <x:v>FAKEISIN0006</x:v>
       </x:c>
-      <x:c r="C16" t="n">
+      <x:c r="D16" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D16" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="E16" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -671,18 +684,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J16" t="str">
+      <x:c r="K16" t="str">
         <x:v>Long</x:v>
       </x:c>
-      <x:c r="K16" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="L16" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N16" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -696,52 +712,56 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="str">
+      <x:c r="A1"/>
+      <x:c r="B1" t="str">
         <x:v>FAKE TEST LEDGER</x:v>
       </x:c>
-      <x:c r="B1"/>
       <x:c r="C1"/>
       <x:c r="D1"/>
+      <x:c r="E1"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
+      <x:c r="A2"/>
+      <x:c r="B2" t="str">
         <x:v>Particulars</x:v>
       </x:c>
-      <x:c r="B2" t="str">
+      <x:c r="C2" t="str">
         <x:v>Posting Date</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="D2" t="str">
         <x:v>Debit</x:v>
       </x:c>
-      <x:c r="D2" t="str">
+      <x:c r="E2" t="str">
         <x:v>Credit</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="str">
+      <x:c r="A3"/>
+      <x:c r="B3" t="str">
         <x:v>Delayed payment charges</x:v>
       </x:c>
-      <x:c r="B3" t="str">
+      <x:c r="C3" t="str">
         <x:v>2026-10-01</x:v>
       </x:c>
-      <x:c r="C3" t="n">
+      <x:c r="D3" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="D3" t="n">
+      <x:c r="E3" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="str">
+      <x:c r="A4"/>
+      <x:c r="B4" t="str">
         <x:v>Unrelated ledger entry</x:v>
       </x:c>
-      <x:c r="B4" t="str">
+      <x:c r="C4" t="str">
         <x:v>2026-10-02</x:v>
       </x:c>
-      <x:c r="C4" t="n">
+      <x:c r="D4" t="n">
         <x:v>999</x:v>
       </x:c>
-      <x:c r="D4" t="n">
+      <x:c r="E4" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>